<commit_message>
Add catch and consumption mean-TE variants and refresh PPR graphs
</commit_message>
<xml_diff>
--- a/PPREstimation/output/top10/077HS_1_Eastern_tropical_Pacific_(1993-1997).xlsx
+++ b/PPREstimation/output/top10/077HS_1_Eastern_tropical_Pacific_(1993-1997).xlsx
@@ -617,7 +617,6 @@
           <t>Import</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>1</v>
       </c>
@@ -701,7 +700,6 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>1</v>
       </c>
@@ -785,7 +783,6 @@
           <t>PP</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
         <v>1</v>
       </c>
@@ -869,7 +866,6 @@
           <t>PP</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
         <v>1</v>
       </c>
@@ -953,7 +949,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
         <v>2</v>
       </c>
@@ -1037,7 +1032,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
         <v>2.696</v>
       </c>
@@ -1121,7 +1115,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
         <v>3.461087778136076</v>
       </c>
@@ -1205,7 +1198,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
         <v>4.39991615849631</v>
       </c>
@@ -1289,7 +1281,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" s="2" t="n">
         <v>3.44544</v>
       </c>
@@ -1373,7 +1364,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" s="2" t="n">
         <v>3.185318165511125</v>
       </c>
@@ -1457,7 +1447,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" s="2" t="n">
         <v>3.418992</v>
       </c>
@@ -1541,7 +1530,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" s="2" t="n">
         <v>4.321909883925428</v>
       </c>
@@ -1625,7 +1613,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" s="2" t="n">
         <v>5.169275633281224</v>
       </c>
@@ -1709,7 +1696,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" s="2" t="n">
         <v>4.582797335097288</v>
       </c>
@@ -1793,7 +1779,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" s="2" t="n">
         <v>4.684856162430195</v>
       </c>
@@ -1877,7 +1862,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" s="2" t="n">
         <v>4.420664237578483</v>
       </c>
@@ -1961,7 +1945,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
         <v>4.625431441306349</v>
       </c>
@@ -2045,7 +2028,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" s="2" t="n">
         <v>4.939615053512908</v>
       </c>
@@ -2129,7 +2111,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" s="2" t="n">
         <v>4.648265802927456</v>
       </c>
@@ -2213,7 +2194,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
         <v>4.565980151254242</v>
       </c>
@@ -2297,7 +2277,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" s="2" t="n">
         <v>2.787816293695809</v>
       </c>
@@ -2381,7 +2360,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" s="2" t="n">
         <v>3.858903435154414</v>
       </c>
@@ -2465,7 +2443,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" s="2" t="n">
         <v>4.60252129055173</v>
       </c>
@@ -2549,7 +2526,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" s="2" t="n">
         <v>4.569097112769175</v>
       </c>
@@ -2633,7 +2609,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" s="2" t="n">
         <v>3.684047921658288</v>
       </c>
@@ -2717,7 +2692,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" s="2" t="n">
         <v>4.925737054707356</v>
       </c>
@@ -2801,7 +2775,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" s="2" t="n">
         <v>4.881898732301488</v>
       </c>
@@ -2885,7 +2858,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" s="2" t="n">
         <v>4.611340694101608</v>
       </c>
@@ -2969,7 +2941,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" s="2" t="n">
         <v>4.943244527650417</v>
       </c>
@@ -3053,7 +3024,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" s="2" t="n">
         <v>4.905973270102381</v>
       </c>
@@ -3137,7 +3107,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" s="2" t="n">
         <v>5.31041244972341</v>
       </c>
@@ -3221,7 +3190,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="n">
         <v>5.166747078644066</v>
       </c>
@@ -3305,7 +3273,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="n">
         <v>4.65346743893112</v>
       </c>
@@ -3389,7 +3356,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="n">
         <v>3.621794494013979</v>
       </c>
@@ -3473,7 +3439,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="n">
         <v>4.64558861514379</v>
       </c>
@@ -3557,7 +3522,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="n">
         <v>5.032080918164987</v>
       </c>
@@ -3641,7 +3605,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="n">
         <v>5.215910779312956</v>
       </c>
@@ -3725,7 +3688,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="n">
         <v>3.805752876269732</v>
       </c>
@@ -3809,7 +3771,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="n">
         <v>3.764337908275556</v>
       </c>
@@ -3893,7 +3854,6 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="n">
         <v>4.751954163749264</v>
       </c>
@@ -3969,7 +3929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4107,6 +4067,16 @@
           <t>MC_new_TE_EEfix</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>SPPR_1995_TEmean_catch</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Ulanowicz_globalTEmean_catch</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -4117,9 +4087,6 @@
           <t>diet_import</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
@@ -4150,19 +4117,18 @@
       <c r="O2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -4173,9 +4139,6 @@
           <t>Detritus</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" s="2" t="n">
         <v>0</v>
       </c>
@@ -4224,7 +4187,9 @@
       <c r="U3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -4235,9 +4200,6 @@
           <t>Small producers</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" s="2" t="n">
         <v>1</v>
       </c>
@@ -4286,7 +4248,9 @@
       <c r="U4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="X4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -4297,9 +4261,6 @@
           <t>Large phytoplankton</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" s="2" t="n">
         <v>1</v>
       </c>
@@ -4348,7 +4309,9 @@
       <c r="U5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -4359,11 +4322,8 @@
           <t>Microzooplankton</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" s="2" t="n">
-        <v>19.0384752574556</v>
+        <v>4.446089013058017</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4.281432852861424</v>
@@ -4410,7 +4370,9 @@
       <c r="U6" s="2" t="n">
         <v>4.212516077220783</v>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="X6" t="n">
+        <v>19.0384752574556</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -4421,11 +4383,8 @@
           <t>Mesozooplankton</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" s="2" t="n">
-        <v>258.0623204078759</v>
+        <v>15.10993548834614</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>15.09134772790235</v>
@@ -4472,7 +4431,9 @@
       <c r="U7" s="2" t="n">
         <v>10.01538138235641</v>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="X7" t="n">
+        <v>258.0623204078759</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -4483,11 +4444,8 @@
           <t>Crabs</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" s="2" t="n">
-        <v>11345.91735421774</v>
+        <v>68.93744071449068</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>52.28254560739003</v>
@@ -4534,7 +4492,9 @@
       <c r="U8" s="2" t="n">
         <v>45.31324285999567</v>
       </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="X8" t="n">
+        <v>11345.91735421774</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -4545,11 +4505,8 @@
           <t>Cephalopods</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" s="2" t="n">
-        <v>46418.39825594125</v>
+        <v>157.6108604371649</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>185.6105489915783</v>
@@ -4596,7 +4553,9 @@
       <c r="U9" s="2" t="n">
         <v>262.5296645598756</v>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="X9" t="n">
+        <v>46418.39825594125</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -4607,11 +4566,8 @@
           <t>Misc. mesopelagic fishes</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" s="2" t="n">
-        <v>3274.879259705181</v>
+        <v>50.11165032849345</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>65.24142741487931</v>
@@ -4658,7 +4614,9 @@
       <c r="U10" s="2" t="n">
         <v>42.85977812755402</v>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="X10" t="n">
+        <v>3274.879259705181</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -4669,11 +4627,8 @@
           <t>Misc. epipelagic fishes</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" s="2" t="n">
-        <v>2439.02620972183</v>
+        <v>38.33473203328829</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>47.0509365833674</v>
@@ -4720,7 +4675,9 @@
       <c r="U11" s="2" t="n">
         <v>41.62038483319467</v>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="X11" t="n">
+        <v>2439.02620972183</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -4731,11 +4688,8 @@
           <t>Flyingfishes</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" s="2" t="n">
-        <v>3101.954576355331</v>
+        <v>48.30997872376624</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>101.7383923527084</v>
@@ -4782,7 +4736,9 @@
       <c r="U12" s="2" t="n">
         <v>69.41568763505934</v>
       </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="X12" t="n">
+        <v>3101.954576355331</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -4793,11 +4749,8 @@
           <t>Miscellaneous piscivores</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" s="2" t="n">
-        <v>248293.8662210611</v>
+        <v>255.2973726448377</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>321.7056115293004</v>
@@ -4844,7 +4797,9 @@
       <c r="U13" s="2" t="n">
         <v>426.4246266521095</v>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="X13" t="n">
+        <v>248293.8662210611</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -4855,11 +4810,8 @@
           <t>Small sharks</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" s="2" t="n">
-        <v>4218253.109541594</v>
+        <v>1006.536396134616</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>110770.4176237767</v>
@@ -4906,7 +4858,9 @@
       <c r="U14" s="2" t="n">
         <v>28588.75663651022</v>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="X14" t="n">
+        <v>4218253.109541594</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -4917,11 +4871,8 @@
           <t>Small wahoo</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" s="2" t="n">
-        <v>928934.3542468947</v>
+        <v>395.7347777619572</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1357.329707193471</v>
@@ -4968,7 +4919,9 @@
       <c r="U15" s="2" t="n">
         <v>1473.375737137782</v>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="X15" t="n">
+        <v>928934.3542468947</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -4979,11 +4932,8 @@
           <t>Small dorado</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" s="2" t="n">
-        <v>616266.845533464</v>
+        <v>373.471531944038</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>1163.485705860615</v>
@@ -5030,7 +4980,9 @@
       <c r="U16" s="2" t="n">
         <v>1869.229847102136</v>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>616266.845533464</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -5041,11 +4993,8 @@
           <t>Small swordfish</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" s="2" t="n">
-        <v>219006.6203108405</v>
+        <v>277.0259597077351</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>4280.891152563265</v>
@@ -5092,7 +5041,9 @@
       <c r="U17" s="2" t="n">
         <v>3655.745926740054</v>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="X17" t="n">
+        <v>219006.6203108405</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -5103,11 +5054,8 @@
           <t>Small sailfish</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" s="2" t="n">
-        <v>1432453.600256445</v>
+        <v>446.5701027284001</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>4428.723869082205</v>
@@ -5154,7 +5102,9 @@
       <c r="U18" s="2" t="n">
         <v>4165.193176144154</v>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="X18" t="n">
+        <v>1432453.600256445</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -5165,11 +5115,8 @@
           <t>Small marlins</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" s="2" t="n">
-        <v>3972790.750112601</v>
+        <v>753.9287445836004</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>40022.83790775665</v>
@@ -5216,7 +5163,9 @@
       <c r="U19" s="2" t="n">
         <v>16713.63410362666</v>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="X19" t="n">
+        <v>3972790.750112601</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -5227,11 +5176,8 @@
           <t>Small bigeye tuna</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" s="2" t="n">
-        <v>535778.5472335232</v>
+        <v>390.598342194627</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3323.53436263723</v>
@@ -5278,7 +5224,9 @@
       <c r="U20" s="2" t="n">
         <v>2818.187954263566</v>
       </c>
-      <c r="V20" t="inlineStr"/>
+      <c r="X20" t="n">
+        <v>535778.5472335232</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -5289,11 +5237,8 @@
           <t>Small yellowfin tuna</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" s="2" t="n">
-        <v>293853.6427072483</v>
+        <v>315.3133069095059</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1292.944299665767</v>
@@ -5340,7 +5285,9 @@
       <c r="U21" s="2" t="n">
         <v>1587.205433004437</v>
       </c>
-      <c r="V21" t="inlineStr"/>
+      <c r="X21" t="n">
+        <v>293853.6427072483</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -5351,11 +5298,8 @@
           <t>Bluefin tuna</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" s="2" t="n">
-        <v>140343.5678854656</v>
+        <v>95.25223060127158</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>785.4449092941215</v>
@@ -5402,7 +5346,9 @@
       <c r="U22" s="2" t="n">
         <v>580.8463791332262</v>
       </c>
-      <c r="V22" t="inlineStr"/>
+      <c r="X22" t="n">
+        <v>140343.5678854656</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -5413,11 +5359,8 @@
           <t>Auxis spp.</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" s="2" t="n">
-        <v>42937.12267024055</v>
+        <v>107.5710899752451</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>304.5761627545889</v>
@@ -5464,7 +5407,9 @@
       <c r="U23" s="2" t="n">
         <v>629.6893011147753</v>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="X23" t="n">
+        <v>42937.12267024055</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -5475,11 +5420,8 @@
           <t>Albacore</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" s="2" t="n">
-        <v>470800.6009548716</v>
+        <v>365.4517211358057</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>3630.458131442678</v>
@@ -5526,7 +5468,9 @@
       <c r="U24" s="2" t="n">
         <v>3867.027617984191</v>
       </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="X24" t="n">
+        <v>470800.6009548716</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -5537,11 +5481,8 @@
           <t>Skipjack tuna</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" s="2" t="n">
-        <v>357889.6618935249</v>
+        <v>350.5865197239083</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>3101.223515491341</v>
@@ -5588,7 +5529,9 @@
       <c r="U25" s="2" t="n">
         <v>1765.352590475814</v>
       </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="X25" t="n">
+        <v>357889.6618935249</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -5599,11 +5542,8 @@
           <t>Rays</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" s="2" t="n">
-        <v>64272.16565522837</v>
+        <v>112.0900056974743</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>1167.961695826983</v>
@@ -5650,7 +5590,9 @@
       <c r="U26" s="2" t="n">
         <v>439.2973513297788</v>
       </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="X26" t="n">
+        <v>64272.16565522837</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -5661,11 +5603,8 @@
           <t>Large sharks</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" s="2" t="n">
-        <v>3702709.932104028</v>
+        <v>807.5749807017626</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>324275.8668348721</v>
@@ -5712,7 +5651,9 @@
       <c r="U27" s="2" t="n">
         <v>49948.29576723443</v>
       </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="X27" t="n">
+        <v>3702709.932104028</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -5723,11 +5664,8 @@
           <t>Large wahoo</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" s="2" t="n">
-        <v>1878276.214472115</v>
+        <v>624.0903464697864</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>56991.36048557569</v>
@@ -5774,7 +5712,9 @@
       <c r="U28" s="2" t="n">
         <v>4531.656138834664</v>
       </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="X28" t="n">
+        <v>1878276.214472115</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -5785,11 +5725,8 @@
           <t>Large dorado</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" s="2" t="n">
-        <v>694840.7758726039</v>
+        <v>363.6617652984876</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>11350.92168873759</v>
@@ -5836,7 +5773,9 @@
       <c r="U29" s="2" t="n">
         <v>3243.218669719786</v>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="X29" t="n">
+        <v>694840.7758726039</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -5847,11 +5786,8 @@
           <t>Large swordfish</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" s="2" t="n">
-        <v>738583.2643352292</v>
+        <v>527.6771719827528</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>4188.650429331983</v>
@@ -5898,7 +5834,9 @@
       <c r="U30" s="2" t="n">
         <v>4100.86669899936</v>
       </c>
-      <c r="V30" t="inlineStr"/>
+      <c r="X30" t="n">
+        <v>738583.2643352292</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -5909,11 +5847,8 @@
           <t>Large sailfish</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" s="2" t="n">
-        <v>3377289.487015368</v>
+        <v>703.2339519243473</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>23040.99652905024</v>
@@ -5960,7 +5895,9 @@
       <c r="U31" s="2" t="n">
         <v>3809.582483935851</v>
       </c>
-      <c r="V31" t="inlineStr"/>
+      <c r="X31" t="n">
+        <v>3377289.487015368</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -5971,11 +5908,8 @@
           <t>Large marlins</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" s="2" t="n">
-        <v>5293328.249140459</v>
+        <v>1139.916644518609</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>79425.16999386242</v>
@@ -6022,7 +5956,9 @@
       <c r="U32" s="2" t="n">
         <v>16684.06127666681</v>
       </c>
-      <c r="V32" t="inlineStr"/>
+      <c r="X32" t="n">
+        <v>5293328.249140459</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -6033,11 +5969,8 @@
           <t>Large bigeye tuna</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" s="2" t="n">
-        <v>967475.5603432835</v>
+        <v>624.3690770421446</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>8999.590696702575</v>
@@ -6084,7 +6017,9 @@
       <c r="U33" s="2" t="n">
         <v>4191.396248402105</v>
       </c>
-      <c r="V33" t="inlineStr"/>
+      <c r="X33" t="n">
+        <v>967475.5603432835</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -6095,11 +6030,8 @@
           <t>Large yellowfin tuna</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" s="2" t="n">
-        <v>674379.9357057333</v>
+        <v>394.1801387969149</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>4151.993868297915</v>
@@ -6146,7 +6078,9 @@
       <c r="U34" s="2" t="n">
         <v>2678.686260352696</v>
       </c>
-      <c r="V34" t="inlineStr"/>
+      <c r="X34" t="n">
+        <v>674379.9357057333</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -6157,11 +6091,8 @@
           <t>Sea turtles</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" s="2" t="n">
-        <v>70523.36274842665</v>
+        <v>111.8007151167495</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>1178.701169920576</v>
@@ -6208,7 +6139,9 @@
       <c r="U35" s="2" t="n">
         <v>603.3186870746403</v>
       </c>
-      <c r="V35" t="inlineStr"/>
+      <c r="X35" t="n">
+        <v>70523.36274842665</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -6219,11 +6152,8 @@
           <t>Mesopelagic dolphins</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" s="2" t="n">
-        <v>277983.1118262132</v>
+        <v>338.7356200368008</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>205441.1928062249</v>
@@ -6270,7 +6200,9 @@
       <c r="U36" s="2" t="n">
         <v>43463.2079476054</v>
       </c>
-      <c r="V36" t="inlineStr"/>
+      <c r="X36" t="n">
+        <v>277983.1118262132</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -6281,11 +6213,8 @@
           <t>Spotted dolphin</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="n">
-        <v>776249.4682305149</v>
+        <v>542.9228462249848</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>318805.3951533652</v>
@@ -6332,7 +6261,9 @@
       <c r="U37" s="2" t="n">
         <v>100113.4474141692</v>
       </c>
-      <c r="V37" t="inlineStr"/>
+      <c r="X37" t="n">
+        <v>776249.4682305149</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -6343,11 +6274,8 @@
           <t>Toothed whales</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" s="2" t="n">
-        <v>1798653.453687605</v>
+        <v>721.873948204194</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>-1.048708891161729e+20</v>
@@ -6394,7 +6322,9 @@
       <c r="U38" s="2" t="n">
         <v>148637.1774245259</v>
       </c>
-      <c r="V38" t="inlineStr"/>
+      <c r="X38" t="n">
+        <v>1798653.453687605</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -6405,11 +6335,8 @@
           <t>Baleen whales</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" s="2" t="n">
-        <v>32711.58745339057</v>
+        <v>97.84550742068872</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>11069.47757109662</v>
@@ -6456,7 +6383,9 @@
       <c r="U39" s="2" t="n">
         <v>8974.502194709941</v>
       </c>
-      <c r="V39" t="inlineStr"/>
+      <c r="X39" t="n">
+        <v>32711.58745339057</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -6467,11 +6396,8 @@
           <t>Grazing birds</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" s="2" t="n">
-        <v>23036.73396461979</v>
+        <v>106.7020889677044</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>94541.88556458974</v>
@@ -6518,7 +6444,9 @@
       <c r="U40" s="2" t="n">
         <v>9049.04832068424</v>
       </c>
-      <c r="V40" t="inlineStr"/>
+      <c r="X40" t="n">
+        <v>23036.73396461979</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -6529,11 +6457,8 @@
           <t>Pursuit birds</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" s="2" t="n">
-        <v>347227.7037338472</v>
+        <v>383.059950761719</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>445993.1221813682</v>
@@ -6580,7 +6505,9 @@
       <c r="U41" s="2" t="n">
         <v>112274.8963004638</v>
       </c>
-      <c r="V41" t="inlineStr"/>
+      <c r="X41" t="n">
+        <v>347227.7037338472</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6593,7 +6520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -6731,6 +6658,16 @@
           <t>MC_new_TE_EEfix</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>SPPR_1995_TEmean_catch</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Ulanowicz_globalTEmean_catch</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -6780,19 +6717,21 @@
       <c r="O2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -6860,7 +6799,12 @@
       <c r="U3" s="2" t="n">
         <v>1.778957536312641</v>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -6928,7 +6872,12 @@
       <c r="U4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -6996,7 +6945,12 @@
       <c r="U5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -7014,10 +6968,10 @@
         <v>10</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>19.0384752574556</v>
+        <v>4.446089013058017</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>19.0384752574556</v>
+        <v>4.446089013058017</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4.281432852861424</v>
@@ -7064,7 +7018,12 @@
       <c r="U6" s="2" t="n">
         <v>4.212516077220783</v>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>19.0384752574556</v>
+      </c>
+      <c r="X6" t="n">
+        <v>19.0384752574556</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -7082,10 +7041,10 @@
         <v>49.65923214503357</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>147.9981034209088</v>
+        <v>12.5594594452816</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>258.0623204078759</v>
+        <v>15.10993548834614</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>15.09134772790235</v>
@@ -7132,7 +7091,12 @@
       <c r="U7" s="2" t="n">
         <v>10.01538138235641</v>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="n">
+        <v>147.9981034209088</v>
+      </c>
+      <c r="X7" t="n">
+        <v>258.0623204078759</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -7150,10 +7114,10 @@
         <v>227.9969245087183</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1040.595094499181</v>
+        <v>33.71991503476991</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>11345.91735421774</v>
+        <v>68.93744071449068</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>52.28254560739003</v>
@@ -7200,7 +7164,12 @@
       <c r="U8" s="2" t="n">
         <v>45.31324285999567</v>
       </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="n">
+        <v>1040.595094499181</v>
+      </c>
+      <c r="X8" t="n">
+        <v>11345.91735421774</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -7218,10 +7187,10 @@
         <v>1604.241927407703</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>12634.74293335485</v>
+        <v>119.3836482122332</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46418.39825594125</v>
+        <v>157.6108604371649</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>185.6105489915783</v>
@@ -7268,7 +7237,12 @@
       <c r="U9" s="2" t="n">
         <v>262.5296645598756</v>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>12634.74293335485</v>
+      </c>
+      <c r="X9" t="n">
+        <v>46418.39825594125</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -7286,10 +7260,10 @@
         <v>278.8945322687176</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1346.677732053272</v>
+        <v>38.42303753893232</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3274.879259705181</v>
+        <v>50.11165032849345</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>65.24142741487931</v>
@@ -7336,7 +7310,12 @@
       <c r="U10" s="2" t="n">
         <v>42.85977812755402</v>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>1346.677732053272</v>
+      </c>
+      <c r="X10" t="n">
+        <v>3274.879259705181</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -7354,10 +7333,10 @@
         <v>137.0392256584925</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>542.469666014298</v>
+        <v>24.24536963009198</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>2439.02620972183</v>
+        <v>38.33473203328829</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>47.0509365833674</v>
@@ -7404,7 +7383,12 @@
       <c r="U11" s="2" t="n">
         <v>41.62038483319467</v>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>542.469666014298</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2439.02620972183</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -7422,10 +7406,10 @@
         <v>262.4170203937674</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1245.718652887015</v>
+        <v>36.93634932532552</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3101.954576355331</v>
+        <v>48.30997872376624</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>101.7383923527084</v>
@@ -7472,7 +7456,12 @@
       <c r="U12" s="2" t="n">
         <v>69.41568763505934</v>
       </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>1245.718652887015</v>
+      </c>
+      <c r="X12" t="n">
+        <v>3101.954576355331</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -7490,10 +7479,10 @@
         <v>1724.884841431027</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>13863.16326586525</v>
+        <v>125.1266552778713</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>248293.8662210611</v>
+        <v>255.2973726448377</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>321.7056115293004</v>
@@ -7540,7 +7529,12 @@
       <c r="U13" s="2" t="n">
         <v>426.4246266521095</v>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="n">
+        <v>13863.16326586525</v>
+      </c>
+      <c r="X13" t="n">
+        <v>248293.8662210611</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -7558,10 +7552,10 @@
         <v>12314.63921001886</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>171488.5632349982</v>
+        <v>447.2021618938251</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>4218253.109541594</v>
+        <v>1006.536396134616</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>110770.4176237767</v>
@@ -7608,7 +7602,12 @@
       <c r="U14" s="2" t="n">
         <v>28588.75663651022</v>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>171488.5632349978</v>
+      </c>
+      <c r="X14" t="n">
+        <v>4218253.109541594</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -7626,10 +7625,10 @@
         <v>3286.034793724828</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>31626.18468981195</v>
+        <v>189.9882446821065</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>928934.3542468947</v>
+        <v>395.7347777619572</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1357.329707193471</v>
@@ -7676,7 +7675,12 @@
       <c r="U15" s="2" t="n">
         <v>1473.375737137782</v>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>31626.18468981195</v>
+      </c>
+      <c r="X15" t="n">
+        <v>928934.3542468947</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -7694,10 +7698,10 @@
         <v>3992.979031925721</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40582.19290247135</v>
+        <v>215.5568351536163</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>616266.845533464</v>
+        <v>373.471531944038</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>1163.485705860615</v>
@@ -7744,7 +7748,12 @@
       <c r="U16" s="2" t="n">
         <v>1869.229847102136</v>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="n">
+        <v>40582.19290247135</v>
+      </c>
+      <c r="X16" t="n">
+        <v>616266.845533464</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -7762,10 +7771,10 @@
         <v>2246.436871503071</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>19439.26317612804</v>
+        <v>148.4892571143589</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>219006.6203108405</v>
+        <v>277.0259597077351</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>4280.891152563265</v>
@@ -7812,7 +7821,12 @@
       <c r="U17" s="2" t="n">
         <v>3655.745926740054</v>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>19439.26317612804</v>
+      </c>
+      <c r="X17" t="n">
+        <v>219006.6203108405</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -7830,10 +7844,10 @@
         <v>3780.416091711658</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>37838.5724995039</v>
+        <v>208.0498970498418</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1432453.600256445</v>
+        <v>446.5701027284001</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>4428.723869082205</v>
@@ -7880,7 +7894,12 @@
       <c r="U18" s="2" t="n">
         <v>4165.193176144154</v>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>37838.5724995039</v>
+      </c>
+      <c r="X18" t="n">
+        <v>1432453.600256445</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -7898,10 +7917,10 @@
         <v>7503.818534939922</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>90977.89930520731</v>
+        <v>324.4130252962696</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>3972790.750112601</v>
+        <v>753.9287445836004</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>40022.83790775665</v>
@@ -7948,7 +7967,12 @@
       <c r="U19" s="2" t="n">
         <v>16713.63410362666</v>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>90977.89930520731</v>
+      </c>
+      <c r="X19" t="n">
+        <v>3972790.750112601</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -7966,10 +7990,10 @@
         <v>3581.66891570503</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>35311.97753459433</v>
+        <v>200.8952732065113</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>535778.5472335232</v>
+        <v>390.598342194627</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3323.53436263723</v>
@@ -8016,7 +8040,12 @@
       <c r="U20" s="2" t="n">
         <v>2818.187954263566</v>
       </c>
-      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>35311.97753459433</v>
+      </c>
+      <c r="X20" t="n">
+        <v>535778.5472335232</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -8034,10 +8063,10 @@
         <v>3089.310792137661</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>29223.96593570081</v>
+        <v>182.538331156425</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>293853.6427072483</v>
+        <v>315.3133069095059</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1292.944299665767</v>
@@ -8084,7 +8113,12 @@
       <c r="U21" s="2" t="n">
         <v>1587.205433004437</v>
       </c>
-      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>29223.96593570073</v>
+      </c>
+      <c r="X21" t="n">
+        <v>293853.6427072483</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -8102,10 +8136,10 @@
         <v>53.00088699884484</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>160.86003647511</v>
+        <v>13.10079959838637</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>140343.5678854656</v>
+        <v>95.25223060127158</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>785.4449092941215</v>
@@ -8152,7 +8186,12 @@
       <c r="U22" s="2" t="n">
         <v>580.8463791332262</v>
       </c>
-      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>160.86003647511</v>
+      </c>
+      <c r="X22" t="n">
+        <v>140343.5678854656</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -8170,10 +8209,10 @@
         <v>607.5938584811129</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>3647.549607001933</v>
+        <v>63.63860548444916</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>42937.12267024055</v>
+        <v>107.5710899752451</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>304.5761627545889</v>
@@ -8220,7 +8259,12 @@
       <c r="U23" s="2" t="n">
         <v>629.6893011147753</v>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>3647.549607001933</v>
+      </c>
+      <c r="X23" t="n">
+        <v>42937.12267024055</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -8238,10 +8282,10 @@
         <v>3283.26519345959</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>31592.07908988901</v>
+        <v>189.884468790009</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>470800.6009548716</v>
+        <v>365.4517211358057</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>3630.458131442678</v>
@@ -8288,7 +8332,12 @@
       <c r="U24" s="2" t="n">
         <v>3867.027617984191</v>
       </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="n">
+        <v>31592.07908988901</v>
+      </c>
+      <c r="X24" t="n">
+        <v>470800.6009548716</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -8306,10 +8355,10 @@
         <v>3055.923066318521</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>28820.42176188083</v>
+        <v>181.2575672948874</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>357889.6618935249</v>
+        <v>350.5865197239083</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>3101.223515491341</v>
@@ -8356,7 +8405,12 @@
       <c r="U25" s="2" t="n">
         <v>1765.352590475814</v>
       </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="n">
+        <v>28820.42176188083</v>
+      </c>
+      <c r="X25" t="n">
+        <v>357889.6618935249</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -8374,10 +8428,10 @@
         <v>459.0782072066546</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>2548.213478497368</v>
+        <v>53.06942878590334</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>64272.16565522837</v>
+        <v>112.0900056974743</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>1167.961695826983</v>
@@ -8424,7 +8478,12 @@
       <c r="U26" s="2" t="n">
         <v>439.2973513297788</v>
       </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="n">
+        <v>2548.213478497368</v>
+      </c>
+      <c r="X26" t="n">
+        <v>64272.16565522837</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -8442,10 +8501,10 @@
         <v>7025.669073390927</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>83626.76406771134</v>
+        <v>310.8633946661739</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>3702709.932104028</v>
+        <v>807.5749807017626</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>324275.8668348721</v>
@@ -8492,7 +8551,12 @@
       <c r="U27" s="2" t="n">
         <v>49948.29576723443</v>
       </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="n">
+        <v>83626.76406771156</v>
+      </c>
+      <c r="X27" t="n">
+        <v>3702709.932104028</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -8510,10 +8574,10 @@
         <v>6449.661230973127</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>74955.92220997866</v>
+        <v>294.1011263234942</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1878276.214472115</v>
+        <v>624.0903464697864</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>56991.36048557569</v>
@@ -8560,7 +8624,12 @@
       <c r="U28" s="2" t="n">
         <v>4531.656138834664</v>
       </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="n">
+        <v>74955.92220997886</v>
+      </c>
+      <c r="X28" t="n">
+        <v>1878276.214472115</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -8578,10 +8647,10 @@
         <v>3770.709897219875</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>37714.30050979533</v>
+        <v>207.703612034427</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>694840.7758726039</v>
+        <v>363.6617652984876</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>11350.92168873759</v>
@@ -8628,7 +8697,12 @@
       <c r="U29" s="2" t="n">
         <v>3243.218669719786</v>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="n">
+        <v>37714.30050979533</v>
+      </c>
+      <c r="X29" t="n">
+        <v>694840.7758726039</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -8646,10 +8720,10 @@
         <v>6413.739893605436</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>74422.13529887961</v>
+        <v>293.0386989724674</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>738583.2643352292</v>
+        <v>527.6771719827528</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>4188.650429331983</v>
@@ -8696,7 +8770,12 @@
       <c r="U30" s="2" t="n">
         <v>4100.86669899936</v>
       </c>
-      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="n">
+        <v>74422.13529887961</v>
+      </c>
+      <c r="X30" t="n">
+        <v>738583.2643352292</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -8714,10 +8793,10 @@
         <v>7034.269928039105</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>83757.7904245221</v>
+        <v>311.1099363344255</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>3377289.487015368</v>
+        <v>703.2339519243473</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>23040.99652905024</v>
@@ -8764,7 +8843,12 @@
       <c r="U31" s="2" t="n">
         <v>3809.582483935851</v>
       </c>
-      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="n">
+        <v>83757.7904245221</v>
+      </c>
+      <c r="X31" t="n">
+        <v>3377289.487015368</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -8782,10 +8866,10 @@
         <v>16688.84145028335</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>253018.5490103177</v>
+        <v>544.55271044745</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>5293328.249140459</v>
+        <v>1139.916644518609</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>79425.16999386242</v>
@@ -8832,7 +8916,12 @@
       <c r="U32" s="2" t="n">
         <v>16684.06127666681</v>
       </c>
-      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>253018.549010317</v>
+      </c>
+      <c r="X32" t="n">
+        <v>5293328.249140459</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -8850,10 +8939,10 @@
         <v>10338.00236646424</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>137088.879969405</v>
+        <v>399.2705077620778</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>967475.5603432835</v>
+        <v>624.3690770421446</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>8999.590696702575</v>
@@ -8900,7 +8989,12 @@
       <c r="U33" s="2" t="n">
         <v>4191.396248402105</v>
       </c>
-      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="n">
+        <v>137088.879969405</v>
+      </c>
+      <c r="X33" t="n">
+        <v>967475.5603432835</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -8918,10 +9012,10 @@
         <v>3877.799805094773</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>39090.32497468869</v>
+        <v>211.5070900722843</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>674379.9357057333</v>
+        <v>394.1801387969149</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>4151.993868297915</v>
@@ -8968,7 +9062,12 @@
       <c r="U34" s="2" t="n">
         <v>2678.686260352696</v>
       </c>
-      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="n">
+        <v>39090.32497468869</v>
+      </c>
+      <c r="X34" t="n">
+        <v>674379.9357057333</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -8986,10 +9085,10 @@
         <v>397.4867321858054</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>2119.223935502205</v>
+        <v>48.33973685332538</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>70523.36274842665</v>
+        <v>111.8007151167495</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>1178.701169920576</v>
@@ -9036,7 +9135,12 @@
       <c r="U35" s="2" t="n">
         <v>603.3186870746403</v>
       </c>
-      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="n">
+        <v>2119.223935502205</v>
+      </c>
+      <c r="X35" t="n">
+        <v>70523.36274842665</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -9054,10 +9158,10 @@
         <v>3845.880011464571</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>38679.05404236032</v>
+        <v>210.3773173479493</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>277983.1118262132</v>
+        <v>338.7356200368008</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>205441.1928062249</v>
@@ -9104,7 +9208,12 @@
       <c r="U36" s="2" t="n">
         <v>43463.2079476054</v>
       </c>
-      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="n">
+        <v>38679.05404236032</v>
+      </c>
+      <c r="X36" t="n">
+        <v>277983.1118262132</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -9122,10 +9231,10 @@
         <v>8042.48029271889</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>99417.46006402433</v>
+        <v>339.3183944834912</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>776249.4682305149</v>
+        <v>542.9228462249848</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>318805.3951533652</v>
@@ -9172,7 +9281,12 @@
       <c r="U37" s="2" t="n">
         <v>100113.4474141692</v>
       </c>
-      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="n">
+        <v>99417.46006402433</v>
+      </c>
+      <c r="X37" t="n">
+        <v>776249.4682305149</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -9190,10 +9304,10 @@
         <v>11724.31069383272</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>161040.4631054912</v>
+        <v>433.1912604280295</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1798653.453687605</v>
+        <v>721.873948204194</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>-1.048708891161729e+20</v>
@@ -9240,7 +9354,12 @@
       <c r="U38" s="2" t="n">
         <v>148637.1774245259</v>
       </c>
-      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>161040.4631054912</v>
+      </c>
+      <c r="X38" t="n">
+        <v>1798653.453687605</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -9258,10 +9377,10 @@
         <v>621.801648507611</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3757.048370572718</v>
+        <v>64.59893810159073</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>32711.58745339057</v>
+        <v>97.84550742068872</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>11069.47757109662</v>
@@ -9308,7 +9427,12 @@
       <c r="U39" s="2" t="n">
         <v>8974.502194709941</v>
       </c>
-      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="n">
+        <v>3757.048370572718</v>
+      </c>
+      <c r="X39" t="n">
+        <v>32711.58745339057</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -9326,10 +9450,10 @@
         <v>577.9819086112467</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>3421.639899951951</v>
+        <v>61.61126017568658</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>23036.73396461979</v>
+        <v>106.7020889677044</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>94541.88556458974</v>
@@ -9376,7 +9500,12 @@
       <c r="U40" s="2" t="n">
         <v>9049.04832068424</v>
       </c>
-      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="n">
+        <v>3421.639899951951</v>
+      </c>
+      <c r="X40" t="n">
+        <v>23036.73396461979</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -9394,10 +9523,10 @@
         <v>4801.802536667172</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>51385.82652700003</v>
+        <v>242.9235155667872</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>347227.7037338472</v>
+        <v>383.059950761719</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>445993.1221813682</v>
@@ -9444,7 +9573,12 @@
       <c r="U41" s="2" t="n">
         <v>112274.8963004638</v>
       </c>
-      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="n">
+        <v>51385.82652700003</v>
+      </c>
+      <c r="X41" t="n">
+        <v>347227.7037338472</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9457,7 +9591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -9595,6 +9729,16 @@
           <t>MC_new_TE_EEfix</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>SPPR_1995_TEmean_catch</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Ulanowicz_globalTEmean_catch</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -9644,19 +9788,21 @@
       <c r="O2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P2" t="inlineStr"/>
       <c r="Q2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="n">
+        <v>1</v>
+      </c>
+      <c r="X2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -9724,7 +9870,12 @@
       <c r="U3" s="2" t="n">
         <v>1.778957536312641</v>
       </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
+        <v>1</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -9792,7 +9943,12 @@
       <c r="U4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
+        <v>1</v>
+      </c>
+      <c r="X4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
@@ -9860,7 +10016,12 @@
       <c r="U5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="n">
+        <v>1</v>
+      </c>
+      <c r="X5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
@@ -9878,10 +10039,10 @@
         <v>10</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>19.0384752574556</v>
+        <v>4.446089013058017</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>19.0384752574556</v>
+        <v>4.446089013058017</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>4.281432852861424</v>
@@ -9928,7 +10089,12 @@
       <c r="U6" s="2" t="n">
         <v>4.212516077220783</v>
       </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="n">
+        <v>19.0384752574556</v>
+      </c>
+      <c r="X6" t="n">
+        <v>19.0384752574556</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
@@ -9946,10 +10112,10 @@
         <v>49.65923214503357</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>147.9981034209088</v>
+        <v>12.5594594452816</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>258.0623204078759</v>
+        <v>15.10993548834614</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>15.09134772790235</v>
@@ -9996,7 +10162,12 @@
       <c r="U7" s="2" t="n">
         <v>10.01538138235641</v>
       </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="n">
+        <v>147.9981034209088</v>
+      </c>
+      <c r="X7" t="n">
+        <v>258.0623204078759</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -10014,10 +10185,10 @@
         <v>227.9969245087183</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1040.595094499181</v>
+        <v>33.71991503476991</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>11345.91735421774</v>
+        <v>68.93744071449068</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>52.28254560739003</v>
@@ -10064,7 +10235,12 @@
       <c r="U8" s="2" t="n">
         <v>45.31324285999567</v>
       </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="n">
+        <v>1040.595094499181</v>
+      </c>
+      <c r="X8" t="n">
+        <v>11345.91735421774</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
@@ -10082,10 +10258,10 @@
         <v>1604.241927407703</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>12634.74293335485</v>
+        <v>119.3836482122332</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46418.39825594125</v>
+        <v>157.6108604371649</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>185.6105489915783</v>
@@ -10132,7 +10308,12 @@
       <c r="U9" s="2" t="n">
         <v>262.5296645598756</v>
       </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="n">
+        <v>12634.74293335485</v>
+      </c>
+      <c r="X9" t="n">
+        <v>46418.39825594125</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -10150,10 +10331,10 @@
         <v>278.8945322687176</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1346.677732053272</v>
+        <v>38.42303753893232</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>3274.879259705181</v>
+        <v>50.11165032849345</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>65.24142741487931</v>
@@ -10200,7 +10381,12 @@
       <c r="U10" s="2" t="n">
         <v>42.85977812755402</v>
       </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="n">
+        <v>1346.677732053272</v>
+      </c>
+      <c r="X10" t="n">
+        <v>3274.879259705181</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -10218,10 +10404,10 @@
         <v>137.0392256584925</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>542.469666014298</v>
+        <v>24.24536963009198</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>2439.02620972183</v>
+        <v>38.33473203328829</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>47.0509365833674</v>
@@ -10268,7 +10454,12 @@
       <c r="U11" s="2" t="n">
         <v>41.62038483319467</v>
       </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="n">
+        <v>542.469666014298</v>
+      </c>
+      <c r="X11" t="n">
+        <v>2439.02620972183</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
@@ -10286,10 +10477,10 @@
         <v>262.4170203937674</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1245.718652887015</v>
+        <v>36.93634932532552</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3101.954576355331</v>
+        <v>48.30997872376624</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>101.7383923527084</v>
@@ -10336,7 +10527,12 @@
       <c r="U12" s="2" t="n">
         <v>69.41568763505934</v>
       </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="n">
+        <v>1245.718652887015</v>
+      </c>
+      <c r="X12" t="n">
+        <v>3101.954576355331</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
@@ -10354,10 +10550,10 @@
         <v>1724.884841431027</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>13863.16326586525</v>
+        <v>125.1266552778713</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>248293.8662210611</v>
+        <v>255.2973726448377</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>321.7056115293004</v>
@@ -10404,7 +10600,12 @@
       <c r="U13" s="2" t="n">
         <v>426.4817793444857</v>
       </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="n">
+        <v>13863.16326586525</v>
+      </c>
+      <c r="X13" t="n">
+        <v>248293.8662210611</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -10422,10 +10623,10 @@
         <v>12314.63921001886</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>171488.5632349982</v>
+        <v>447.2021618938251</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>4218255.143063679</v>
+        <v>1006.647298516106</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>110774.2033739881</v>
@@ -10472,7 +10673,12 @@
       <c r="U14" s="2" t="n">
         <v>28591.62163410584</v>
       </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="n">
+        <v>171488.5632349978</v>
+      </c>
+      <c r="X14" t="n">
+        <v>4218255.143063679</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -10490,10 +10696,10 @@
         <v>3286.034793724828</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>31626.18468981195</v>
+        <v>189.9882446821065</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>928934.3542468947</v>
+        <v>395.7347777619572</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1357.329707193471</v>
@@ -10540,7 +10746,12 @@
       <c r="U15" s="2" t="n">
         <v>1473.417334245416</v>
       </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="n">
+        <v>31626.18468981195</v>
+      </c>
+      <c r="X15" t="n">
+        <v>928934.3542468947</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -10558,10 +10769,10 @@
         <v>3992.979031925721</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>40582.19290247135</v>
+        <v>215.5568351536163</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>616266.845533464</v>
+        <v>373.471531944038</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>1163.485705860615</v>
@@ -10608,7 +10819,12 @@
       <c r="U16" s="2" t="n">
         <v>1869.288535289283</v>
       </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="n">
+        <v>40582.19290247135</v>
+      </c>
+      <c r="X16" t="n">
+        <v>616266.845533464</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -10626,10 +10842,10 @@
         <v>2246.436871503071</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>19439.26317612804</v>
+        <v>148.4892571143589</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>219006.6203108405</v>
+        <v>277.0259597077351</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>4280.891152563265</v>
@@ -10676,7 +10892,12 @@
       <c r="U17" s="2" t="n">
         <v>3655.745926740054</v>
       </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="n">
+        <v>19439.26317612804</v>
+      </c>
+      <c r="X17" t="n">
+        <v>219006.6203108405</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -10694,10 +10915,10 @@
         <v>3780.416091711658</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>37838.5724995039</v>
+        <v>208.0498970498418</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>1432453.600256445</v>
+        <v>446.5701027284001</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>4428.723869082205</v>
@@ -10744,7 +10965,12 @@
       <c r="U18" s="2" t="n">
         <v>4165.343069769592</v>
       </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="n">
+        <v>37838.5724995039</v>
+      </c>
+      <c r="X18" t="n">
+        <v>1432453.600256445</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
@@ -10762,10 +10988,10 @@
         <v>7503.818534939922</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>90977.89930520731</v>
+        <v>324.4130252962696</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>3972791.28953558</v>
+        <v>753.9420312160514</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>40025.25320189798</v>
@@ -10812,7 +11038,12 @@
       <c r="U19" s="2" t="n">
         <v>16714.70603931426</v>
       </c>
-      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="n">
+        <v>90977.89930520731</v>
+      </c>
+      <c r="X19" t="n">
+        <v>3972791.28953558</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -10830,10 +11061,10 @@
         <v>3581.66891570503</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>35311.97753459433</v>
+        <v>200.8952732065113</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>535778.5472335232</v>
+        <v>390.598342194627</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>3323.53436263723</v>
@@ -10880,7 +11111,12 @@
       <c r="U20" s="2" t="n">
         <v>2818.245628243397</v>
       </c>
-      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="n">
+        <v>35311.97753459433</v>
+      </c>
+      <c r="X20" t="n">
+        <v>535778.5472335232</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -10898,10 +11134,10 @@
         <v>3089.310792137661</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>29223.96593570081</v>
+        <v>182.538331156425</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>293853.6427072483</v>
+        <v>315.3133069095059</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>1292.944299665767</v>
@@ -10948,7 +11184,12 @@
       <c r="U21" s="2" t="n">
         <v>1587.355915142449</v>
       </c>
-      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="n">
+        <v>29223.96593570073</v>
+      </c>
+      <c r="X21" t="n">
+        <v>293853.6427072483</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
@@ -10966,10 +11207,10 @@
         <v>53.00088699884484</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>160.86003647511</v>
+        <v>13.10079959838637</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>140356.2665484623</v>
+        <v>98.21777197298127</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>801.9874398114631</v>
@@ -11016,7 +11257,12 @@
       <c r="U22" s="2" t="n">
         <v>594.1382322445124</v>
       </c>
-      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="n">
+        <v>160.86003647511</v>
+      </c>
+      <c r="X22" t="n">
+        <v>140356.2665484623</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
@@ -11034,10 +11280,10 @@
         <v>607.5938584811129</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>3647.549607001933</v>
+        <v>63.63860548444916</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>42937.12267024055</v>
+        <v>107.5710899752451</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>304.5761627545889</v>
@@ -11084,7 +11330,12 @@
       <c r="U23" s="2" t="n">
         <v>629.6926029617887</v>
       </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="n">
+        <v>3647.549607001933</v>
+      </c>
+      <c r="X23" t="n">
+        <v>42937.12267024055</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
@@ -11102,10 +11353,10 @@
         <v>3283.26519345959</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>31592.07908988901</v>
+        <v>189.884468790009</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>470800.6009548716</v>
+        <v>365.4517211358057</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>3630.458131442678</v>
@@ -11152,7 +11403,12 @@
       <c r="U24" s="2" t="n">
         <v>3867.069252864634</v>
       </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="n">
+        <v>31592.07908988901</v>
+      </c>
+      <c r="X24" t="n">
+        <v>470800.6009548716</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -11170,10 +11426,10 @@
         <v>3055.923066318521</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>28820.42176188083</v>
+        <v>181.2575672948874</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>357889.6618935249</v>
+        <v>350.5865197239083</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>3101.223515491341</v>
@@ -11220,7 +11476,12 @@
       <c r="U25" s="2" t="n">
         <v>1765.357273815645</v>
       </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="n">
+        <v>28820.42176188083</v>
+      </c>
+      <c r="X25" t="n">
+        <v>357889.6618935249</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
@@ -11238,10 +11499,10 @@
         <v>459.0782072066546</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>2548.213478497368</v>
+        <v>53.06942878590334</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>64272.16565522837</v>
+        <v>112.0900056974743</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>1167.961695826983</v>
@@ -11288,7 +11549,12 @@
       <c r="U26" s="2" t="n">
         <v>439.2973513297788</v>
       </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="n">
+        <v>2548.213478497368</v>
+      </c>
+      <c r="X26" t="n">
+        <v>64272.16565522837</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
@@ -11306,10 +11572,10 @@
         <v>7025.669073390927</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>83626.76406771134</v>
+        <v>310.8633946661739</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>3702710.492467787</v>
+        <v>807.6021142637799</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>324278.0743925797</v>
@@ -11356,7 +11622,12 @@
       <c r="U27" s="2" t="n">
         <v>49949.64473744722</v>
       </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="n">
+        <v>83626.76406771156</v>
+      </c>
+      <c r="X27" t="n">
+        <v>3702710.492467787</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -11374,10 +11645,10 @@
         <v>6449.661230973127</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>74955.92220997866</v>
+        <v>294.1011263234942</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>1878276.939761659</v>
+        <v>624.1299016525179</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>56997.32066201209</v>
@@ -11424,7 +11695,12 @@
       <c r="U28" s="2" t="n">
         <v>4532.180664513754</v>
       </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="n">
+        <v>74955.92220997886</v>
+      </c>
+      <c r="X28" t="n">
+        <v>1878276.939761659</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
@@ -11442,10 +11718,10 @@
         <v>3770.709897219875</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>37714.30050979533</v>
+        <v>207.703612034427</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>694841.0176357852</v>
+        <v>363.6749503593981</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>11352.12929346536</v>
@@ -11492,7 +11768,12 @@
       <c r="U29" s="2" t="n">
         <v>3243.577911431544</v>
       </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="n">
+        <v>37714.30050979533</v>
+      </c>
+      <c r="X29" t="n">
+        <v>694841.0176357852</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
@@ -11510,10 +11791,10 @@
         <v>6413.739893605436</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>74422.13529887961</v>
+        <v>293.0386989724674</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>738583.5115368461</v>
+        <v>527.6906536401256</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>4189.050230218255</v>
@@ -11560,7 +11841,12 @@
       <c r="U30" s="2" t="n">
         <v>4101.172055549826</v>
       </c>
-      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="n">
+        <v>74422.13529887961</v>
+      </c>
+      <c r="X30" t="n">
+        <v>738583.5115368461</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
@@ -11578,10 +11864,10 @@
         <v>7034.269928039105</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>83757.7904245221</v>
+        <v>311.1099363344255</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>3377289.604814772</v>
+        <v>703.2351013343957</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>23042.10822258391</v>
@@ -11628,7 +11914,12 @@
       <c r="U31" s="2" t="n">
         <v>3809.777878065222</v>
       </c>
-      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="n">
+        <v>83757.7904245221</v>
+      </c>
+      <c r="X31" t="n">
+        <v>3377289.604814772</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
@@ -11646,10 +11937,10 @@
         <v>16688.84145028335</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>253018.5490103177</v>
+        <v>544.55271044745</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>5293329.843124549</v>
+        <v>1139.997222690914</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>79427.00194000766</v>
@@ -11696,7 +11987,12 @@
       <c r="U32" s="2" t="n">
         <v>16685.11395647036</v>
       </c>
-      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="n">
+        <v>253018.549010317</v>
+      </c>
+      <c r="X32" t="n">
+        <v>5293329.843124549</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
@@ -11714,10 +12010,10 @@
         <v>10338.00236646424</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>137088.879969405</v>
+        <v>399.2705077620778</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>967475.5603432835</v>
+        <v>624.3690770421446</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>8999.590696702575</v>
@@ -11764,7 +12060,12 @@
       <c r="U33" s="2" t="n">
         <v>4191.461231455989</v>
       </c>
-      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="n">
+        <v>137088.879969405</v>
+      </c>
+      <c r="X33" t="n">
+        <v>967475.5603432835</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
@@ -11782,10 +12083,10 @@
         <v>3877.799805094773</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>39090.32497468869</v>
+        <v>211.5070900722843</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>674380.1774689145</v>
+        <v>394.1933238578254</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>4152.298907867738</v>
@@ -11832,7 +12133,12 @@
       <c r="U34" s="2" t="n">
         <v>2678.797180643298</v>
       </c>
-      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="n">
+        <v>39090.32497468869</v>
+      </c>
+      <c r="X34" t="n">
+        <v>674380.1774689145</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
@@ -11850,10 +12156,10 @@
         <v>397.4867321858054</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>2119.223935502205</v>
+        <v>48.33973685332538</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>70523.36274842665</v>
+        <v>111.8007151167495</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>1178.701169920576</v>
@@ -11900,7 +12206,12 @@
       <c r="U35" s="2" t="n">
         <v>603.3186870746403</v>
       </c>
-      <c r="V35" t="inlineStr"/>
+      <c r="W35" t="n">
+        <v>2119.223935502205</v>
+      </c>
+      <c r="X35" t="n">
+        <v>70523.36274842665</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
@@ -11918,10 +12229,10 @@
         <v>3845.880011464571</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>38679.05404236032</v>
+        <v>210.3773173479493</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>277983.1118262132</v>
+        <v>338.7356200368008</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>205441.1928062249</v>
@@ -11968,7 +12279,12 @@
       <c r="U36" s="2" t="n">
         <v>43463.22168675972</v>
       </c>
-      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="n">
+        <v>38679.05404236032</v>
+      </c>
+      <c r="X36" t="n">
+        <v>277983.1118262132</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
@@ -11986,10 +12302,10 @@
         <v>8042.48029271889</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>99417.46006402433</v>
+        <v>339.3183944834912</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>776249.4682305149</v>
+        <v>542.9228462249848</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>318805.3951533652</v>
@@ -12036,7 +12352,12 @@
       <c r="U37" s="2" t="n">
         <v>100114.0495898625</v>
       </c>
-      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="n">
+        <v>99417.46006402433</v>
+      </c>
+      <c r="X37" t="n">
+        <v>776249.4682305149</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
@@ -12054,10 +12375,10 @@
         <v>11724.31069383272</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>161040.4631054912</v>
+        <v>433.1912604280295</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1798653.695450787</v>
+        <v>721.8871332651045</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>-1.048751108357817e+20</v>
@@ -12104,7 +12425,12 @@
       <c r="U38" s="2" t="n">
         <v>148644.004187067</v>
       </c>
-      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="n">
+        <v>161040.4631054912</v>
+      </c>
+      <c r="X38" t="n">
+        <v>1798653.695450787</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
@@ -12122,10 +12448,10 @@
         <v>621.801648507611</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3757.048370572718</v>
+        <v>64.59893810159073</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>32711.58745339057</v>
+        <v>97.84550742068872</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>11069.47757109662</v>
@@ -12172,7 +12498,12 @@
       <c r="U39" s="2" t="n">
         <v>8974.502194709941</v>
       </c>
-      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="n">
+        <v>3757.048370572718</v>
+      </c>
+      <c r="X39" t="n">
+        <v>32711.58745339057</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
@@ -12190,10 +12521,10 @@
         <v>577.9819086112467</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>3421.639899951951</v>
+        <v>61.61126017568658</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>23036.73396461979</v>
+        <v>106.7020889677044</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>94541.88556458974</v>
@@ -12240,7 +12571,12 @@
       <c r="U40" s="2" t="n">
         <v>9049.04832068424</v>
       </c>
-      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="n">
+        <v>3421.639899951951</v>
+      </c>
+      <c r="X40" t="n">
+        <v>23036.73396461979</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
@@ -12258,10 +12594,10 @@
         <v>4801.802536667172</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>51385.82652700003</v>
+        <v>242.9235155667872</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>347227.7037338472</v>
+        <v>383.059950761719</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>445993.1221813682</v>
@@ -12308,7 +12644,12 @@
       <c r="U41" s="2" t="n">
         <v>112274.8963004638</v>
       </c>
-      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="n">
+        <v>51385.82652700003</v>
+      </c>
+      <c r="X41" t="n">
+        <v>347227.7037338472</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12779,7 +13120,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr"/>
       <c r="AD2" s="2" t="n">
         <v>0</v>
       </c>
@@ -12905,7 +13245,6 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
           <t>Eastern_tropical_Pacific (1993-1997)</t>
@@ -12969,7 +13308,6 @@
           <t>FAIL</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr"/>
       <c r="AD3" s="2" t="n">
         <v>0</v>
       </c>
@@ -13163,7 +13501,6 @@
           <t>OK</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr"/>
       <c r="AD4" s="2" t="n">
         <v>0</v>
       </c>
@@ -13265,7 +13602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13326,14 +13663,12 @@
       <c r="C2" s="2" t="n">
         <v>64.95710523456431</v>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" s="2" t="n">
         <v>554.122932</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.1172250803627891</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -13347,14 +13682,12 @@
       <c r="C3" s="2" t="n">
         <v>75.12531376914126</v>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" s="2" t="n">
         <v>554.122932</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>0.1355751755264683</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -13363,19 +13696,17 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>841.7151483924245</v>
+        <v>3.730744646298155</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>841.7151483924245</v>
-      </c>
-      <c r="D4" t="inlineStr"/>
+        <v>3.730744646298155</v>
+      </c>
       <c r="E4" s="2" t="n">
         <v>554.122932</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>1.519004357669183</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+        <v>0.006732702133139935</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -13384,22 +13715,22 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10895.74325920673</v>
+        <v>6.772994308333213</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10895.74066787679</v>
+        <v>6.77275249352762</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>10895.74066787679</v>
+        <v>6.77275249352762</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>554.122932</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>19.66303872057906</v>
+        <v>0.01222247285287883</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>19.66303872057906</v>
+        <v>0.01222247285287883</v>
       </c>
     </row>
     <row r="6">
@@ -13800,6 +14131,50 @@
       </c>
       <c r="G21" s="2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SPPR_1995_TEmean_catch</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>841.7151483924241</v>
+      </c>
+      <c r="C22" t="n">
+        <v>841.7151483924241</v>
+      </c>
+      <c r="E22" t="n">
+        <v>554.122932</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1.519004357669183</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ulanowicz_globalTEmean_catch</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>10895.74325920673</v>
+      </c>
+      <c r="C23" t="n">
+        <v>10895.74066787679</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10895.74066787679</v>
+      </c>
+      <c r="E23" t="n">
+        <v>554.122932</v>
+      </c>
+      <c r="F23" t="n">
+        <v>19.66303872057906</v>
+      </c>
+      <c r="G23" t="n">
+        <v>19.66303872057906</v>
       </c>
     </row>
   </sheetData>
@@ -13935,7 +14310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13971,7 +14346,6 @@
           <t>NaN means not available, never zero. A basal source a method does not resolve is NaN, and a method that raised leaves its entire block NaN.</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -13984,7 +14358,6 @@
           <t>sppr_all, sppr_inner and sppr_PP are the same table under three source scopes, mirroring get_PPR: sppr_all sums every basal source, sppr_inner drops Import, and sppr_PP drops Import and Detritus. Each is a flat groups x methods table -- rows are group seq with the group name in the first column, one column per method, no MultiIndex. Sums are taken over each method's own basal-source columns before aggregation; the per-source breakdown itself is not written to the workbook.</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -13997,7 +14370,6 @@
           <t>SPPR_1986 and SPPR_1995 return one un-attributed SPPR column, so their value cannot be split into a PP-only part: they are NaN in sppr_PP (and in ppr_pp_only) while sppr_inner and sppr_all carry the total. A method that resolves no Detritus source (SPPR_2015) has sppr_inner equal to sppr_PP by construction.</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -14010,7 +14382,6 @@
           <t>SPPR_2015() has no only_pp_det parameter (only_pp belongs to get_PPR / get_PPR2NPP_ratio). It is called bare here and PP-only filtering is applied downstream at the get_PPR layer, which is what the ppr_pp_only column and SUM_PP already do.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -14023,7 +14394,6 @@
           <t>Under det_open_mode='none' det_theta does not affect the recycling gain b at all (verified: identical b at theta = 1, 3 and 10). Do not read the health sheet as a theta sensitivity.</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -14036,7 +14406,6 @@
           <t>MC runs use exclude_diverged=True, so draws graded FAIL on divergence are dropped as well as draws with a negative SPPR. The two are often the same draws rather than additive -- see the mc_diagnostics sheet for the split by cause.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -14049,7 +14418,6 @@
           <t>SPPR_EwE and the Monte-Carlo methods are called with silent=True rather than silent=False: PPRCalculator imports tqdm.notebook, whose bar needs ipywidgets and raises ImportError('IProgress not found') outside Jupyter, which makes those methods fail outright in a terminal run. Nothing is lost -- this exporter has its own progress bar, and the MC rejection counts appear in mc_diagnostics and in the run report.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -14062,7 +14430,6 @@
           <t>diagnose_sppr grades a CONFIGURATION, not a model: a model can be healthy under one TE_option and divergent under another. Read each row with its config_ columns.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -14075,7 +14442,6 @@
           <t>Every SPPR method, and every diagnose_sppr row, runs in a worker process with a wall-clock budget (180 s by default; --timeout SECONDS on the command line, method_timeout= from Python, and None or 0 to disable it). A method still running when the budget expires is killed and left NaN, exactly like a method that raised -- the status column of this sheet and the run report are the only places that say which of the two happened. A timeout is a statement about this machine and this model, not about the method: rerun it with a larger budget before reading anything into it.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -14119,7 +14485,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Christensen &amp; Pauly (1995): per-group TE^(1-TL) with global_TE='mean'.</t>
+          <t>Pauly &amp; Christensen (1995): per-group TE^(1-TL) with global_TE='mean'. Arithmetic mean with consumer consumption weights.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -14136,7 +14502,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nullspace form of the EwE path sum, global TE at the true mean (Jensen-able on TL).</t>
+          <t>Nullspace form of the EwE path sum, global TE at the consumer consumption-weighted arithmetic mean (Jensen-able on TL).</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -14412,6 +14778,40 @@
         </is>
       </c>
       <c r="C30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>method: SPPR_1995_TEmean_catch</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Pauly &amp; Christensen (1995): per-group TE^(1-TL) with global_TE='mean'. Arithmetic mean with consumer catch weights. Consumer biomass fallback when consumer catch is zero.</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>method: Ulanowicz_globalTEmean_catch</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Nullspace form of the EwE path sum, global TE at the consumer catch-weighted arithmetic mean. Consumer biomass fallback when consumer catch is zero (Jensen-able on TL).</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>